<commit_message>
clean, narrow cal format
</commit_message>
<xml_diff>
--- a/data/PSUE_Schiesskalender2026.xlsx
+++ b/data/PSUE_Schiesskalender2026.xlsx
@@ -1,24 +1,24 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="P:\01. Michael\05. Pistolensektion Unterengstringen\psue_admin\Anlässe\Schiesskalender\2026\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\stephanw\source\psue_website\shootical\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{411ED397-397D-457A-ACEB-D6B0A6171B00}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1EC48126-C062-4F40-8693-0D19F9AA5031}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3900" yWindow="3900" windowWidth="28800" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="7" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Tabelle1!$A$4:$G$18</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Tabelle1!$A$4:$G$16</definedName>
     <definedName name="Datenschnitt_Aushang">#N/A</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Tabelle1!$A$1:$F$87</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Tabelle1!$A$1:$F$85</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -33,21 +33,12 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="284" uniqueCount="106">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="275" uniqueCount="106">
   <si>
     <t>Tag</t>
   </si>
@@ -394,18 +385,13 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="dd/mm/yy"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="4">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Arial"/>
-      <family val="2"/>
     </font>
     <font>
       <sz val="9"/>
@@ -483,11 +469,11 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -495,20 +481,17 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -526,13 +509,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="a^n_Text" xfId="1" xr:uid="{FCDCEC73-9B25-4C63-99B7-EF3A0921069E}"/>
-    <cellStyle name="Standard" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="15">
     <dxf>
@@ -717,8 +700,8 @@
     <xdr:to>
       <xdr:col>9</xdr:col>
       <xdr:colOff>504825</xdr:colOff>
-      <xdr:row>15</xdr:row>
-      <xdr:rowOff>34925</xdr:rowOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>115988</xdr:rowOff>
     </xdr:to>
     <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer">
       <mc:Choice Requires="sle15">
@@ -805,27 +788,27 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{139EDE26-005F-4C9E-A4C0-934E391B5AC6}" name="Tabelle1" displayName="Tabelle1" ref="A4:G101" totalsRowShown="0" headerRowDxfId="8" dataDxfId="7" headerRowCellStyle="Standard" dataCellStyle="Standard">
-  <autoFilter ref="A4:G101" xr:uid="{139EDE26-005F-4C9E-A4C0-934E391B5AC6}">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{139EDE26-005F-4C9E-A4C0-934E391B5AC6}" name="Tabelle1" displayName="Tabelle1" ref="A4:G99" totalsRowShown="0" headerRowDxfId="8" dataDxfId="7">
+  <autoFilter ref="A4:G99" xr:uid="{139EDE26-005F-4C9E-A4C0-934E391B5AC6}">
     <filterColumn colId="6">
       <filters>
         <filter val="Ja"/>
       </filters>
     </filterColumn>
   </autoFilter>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A5:G101">
-    <sortCondition ref="A4:A101"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A5:G99">
+    <sortCondition ref="A4:A99"/>
   </sortState>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{F6DC726F-B501-48FC-80B8-316D5F6F1776}" name="Datum" dataDxfId="6" dataCellStyle="Standard"/>
-    <tableColumn id="2" xr3:uid="{AFD7064C-A80E-4258-AAED-2F2014CF6851}" name="Tag" dataDxfId="5" dataCellStyle="Standard">
+    <tableColumn id="1" xr3:uid="{F6DC726F-B501-48FC-80B8-316D5F6F1776}" name="Datum" dataDxfId="6"/>
+    <tableColumn id="2" xr3:uid="{AFD7064C-A80E-4258-AAED-2F2014CF6851}" name="Tag" dataDxfId="5">
       <calculatedColumnFormula>TEXT(A5,"TTTT")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{B7AD4EFC-42BF-4546-869A-02B65AD1C65A}" name="Zeit" dataDxfId="4" dataCellStyle="Standard"/>
-    <tableColumn id="4" xr3:uid="{63A7E33E-E558-44E2-B9A2-B6CEC5D08484}" name="Schiessleitung" dataDxfId="3" dataCellStyle="Standard"/>
-    <tableColumn id="5" xr3:uid="{1EF3449F-A7FF-4644-9829-66D5B860F157}" name="Assistent" dataDxfId="2" dataCellStyle="Standard"/>
-    <tableColumn id="6" xr3:uid="{81F6F6EF-DB0C-4BC5-91AC-F20C1C0E01A5}" name="Anlass, Kalenderversion  2026" dataDxfId="1" dataCellStyle="Standard"/>
-    <tableColumn id="7" xr3:uid="{88813096-CC49-4232-8F88-F4D0912FA06B}" name="Aushang" dataDxfId="0" dataCellStyle="Standard"/>
+    <tableColumn id="3" xr3:uid="{B7AD4EFC-42BF-4546-869A-02B65AD1C65A}" name="Zeit" dataDxfId="4"/>
+    <tableColumn id="4" xr3:uid="{63A7E33E-E558-44E2-B9A2-B6CEC5D08484}" name="Schiessleitung" dataDxfId="3"/>
+    <tableColumn id="5" xr3:uid="{1EF3449F-A7FF-4644-9829-66D5B860F157}" name="Assistent" dataDxfId="2"/>
+    <tableColumn id="6" xr3:uid="{81F6F6EF-DB0C-4BC5-91AC-F20C1C0E01A5}" name="Anlass, Kalenderversion  2026" dataDxfId="1"/>
+    <tableColumn id="7" xr3:uid="{88813096-CC49-4232-8F88-F4D0912FA06B}" name="Aushang" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="ENP" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1098,29 +1081,29 @@
     <tabColor rgb="FF00B0F0"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G101"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="15.7265625" defaultRowHeight="14.5"/>
+  <dimension ref="A1:G99"/>
+  <sheetFormatPr defaultColWidth="15.7109375" defaultRowHeight="18" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="15.7265625" style="12"/>
-    <col min="3" max="3" width="12.7265625" customWidth="1"/>
+    <col min="1" max="1" width="15.7109375" style="11"/>
+    <col min="3" max="3" width="12.7109375" customWidth="1"/>
     <col min="4" max="5" width="16" customWidth="1"/>
-    <col min="6" max="6" width="50.7265625" customWidth="1"/>
-    <col min="7" max="7" width="10.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="50.7109375" customWidth="1"/>
+    <col min="7" max="7" width="10.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="26">
-      <c r="A1" s="14" t="s">
+    <row r="1" spans="1:7" ht="18" customHeight="1">
+      <c r="A1" s="13" t="s">
         <v>83</v>
       </c>
-      <c r="B1" s="14"/>
-      <c r="C1" s="14"/>
-      <c r="D1" s="14"/>
-      <c r="E1" s="14"/>
-      <c r="F1" s="14"/>
-      <c r="G1" s="6"/>
-    </row>
-    <row r="4" spans="1:7">
-      <c r="A4" s="9" t="s">
+      <c r="B1" s="13"/>
+      <c r="C1" s="13"/>
+      <c r="D1" s="13"/>
+      <c r="E1" s="13"/>
+      <c r="F1" s="13"/>
+      <c r="G1" s="5"/>
+    </row>
+    <row r="4" spans="1:7" ht="18" customHeight="1">
+      <c r="A4" s="8" t="s">
         <v>40</v>
       </c>
       <c r="B4" s="1" t="s">
@@ -1142,19 +1125,19 @@
         <v>85</v>
       </c>
     </row>
-    <row r="5" spans="1:7">
-      <c r="A5" s="10">
+    <row r="5" spans="1:7" ht="18" customHeight="1">
+      <c r="A5" s="9">
         <v>46079</v>
       </c>
       <c r="B5" s="1" t="str">
-        <f t="shared" ref="B5:B36" si="0">TEXT(A5,"TTTT")</f>
-        <v>Donnerstag</v>
+        <f t="shared" ref="B5:B34" si="0">TEXT(A5,"TTTT")</f>
+        <v>TTTT</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="D5" s="7"/>
-      <c r="E5" s="7"/>
+      <c r="D5" s="6"/>
+      <c r="E5" s="6"/>
       <c r="F5" s="1" t="s">
         <v>37</v>
       </c>
@@ -1162,13 +1145,13 @@
         <v>87</v>
       </c>
     </row>
-    <row r="6" spans="1:7" hidden="1">
-      <c r="A6" s="10">
+    <row r="6" spans="1:7" ht="18" customHeight="1">
+      <c r="A6" s="9">
         <v>46084</v>
       </c>
       <c r="B6" s="1" t="str">
         <f t="shared" si="0"/>
-        <v>Dienstag</v>
+        <v>TTTT</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>46</v>
@@ -1186,13 +1169,13 @@
         <v>88</v>
       </c>
     </row>
-    <row r="7" spans="1:7" hidden="1">
-      <c r="A7" s="10">
+    <row r="7" spans="1:7" ht="18" customHeight="1">
+      <c r="A7" s="9">
         <v>46087</v>
       </c>
       <c r="B7" s="1" t="str">
         <f t="shared" si="0"/>
-        <v>Freitag</v>
+        <v>TTTT</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>41</v>
@@ -1208,361 +1191,355 @@
         <v>88</v>
       </c>
     </row>
-    <row r="8" spans="1:7">
-      <c r="A8" s="10">
-        <v>46084</v>
+    <row r="8" spans="1:7" ht="18" customHeight="1">
+      <c r="A8" s="9">
+        <v>46090</v>
       </c>
       <c r="B8" s="1" t="str">
         <f t="shared" si="0"/>
-        <v>Dienstag</v>
+        <v>TTTT</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="D8" s="7" t="s">
-        <v>55</v>
-      </c>
-      <c r="E8" s="7" t="s">
-        <v>81</v>
-      </c>
-      <c r="F8" s="3" t="s">
-        <v>45</v>
+        <v>4</v>
+      </c>
+      <c r="D8" s="1"/>
+      <c r="E8" s="1"/>
+      <c r="F8" s="7" t="s">
+        <v>5</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7">
-      <c r="A9" s="10">
-        <v>46087</v>
+        <v>87</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" ht="18" customHeight="1">
+      <c r="A9" s="9">
+        <v>46096</v>
       </c>
       <c r="B9" s="1" t="str">
         <f t="shared" si="0"/>
-        <v>Freitag</v>
+        <v>TTTT</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="D9" s="7" t="s">
-        <v>81</v>
-      </c>
-      <c r="E9" s="7"/>
-      <c r="F9" s="3" t="s">
-        <v>78</v>
+        <v>6</v>
+      </c>
+      <c r="D9" s="6"/>
+      <c r="E9" s="6"/>
+      <c r="F9" s="1" t="s">
+        <v>7</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7">
-      <c r="A10" s="10">
-        <v>46090</v>
+        <v>87</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" ht="18" customHeight="1">
+      <c r="A10" s="9">
+        <v>46097</v>
       </c>
       <c r="B10" s="1" t="str">
         <f t="shared" si="0"/>
-        <v>Montag</v>
+        <v>TTTT</v>
       </c>
       <c r="C10" s="1" t="s">
         <v>4</v>
       </c>
       <c r="D10" s="1"/>
       <c r="E10" s="1"/>
-      <c r="F10" s="8" t="s">
-        <v>5</v>
+      <c r="F10" s="1" t="s">
+        <v>57</v>
       </c>
       <c r="G10" s="1" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="11" spans="1:7">
-      <c r="A11" s="10">
-        <v>46096</v>
+    <row r="11" spans="1:7" ht="18" customHeight="1">
+      <c r="A11" s="9">
+        <v>46099</v>
       </c>
       <c r="B11" s="1" t="str">
         <f t="shared" si="0"/>
-        <v>Sonntag</v>
+        <v>TTTT</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="D11" s="7"/>
-      <c r="E11" s="7"/>
+        <v>17</v>
+      </c>
+      <c r="D11" s="1"/>
+      <c r="E11" s="1"/>
       <c r="F11" s="1" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="G11" s="1" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="12" spans="1:7">
-      <c r="A12" s="10">
-        <v>46097</v>
+    <row r="12" spans="1:7" ht="18" customHeight="1">
+      <c r="A12" s="9">
+        <v>46100</v>
       </c>
       <c r="B12" s="1" t="str">
         <f t="shared" si="0"/>
-        <v>Montag</v>
+        <v>TTTT</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="D12" s="1"/>
-      <c r="E12" s="1"/>
+        <v>27</v>
+      </c>
+      <c r="D12" s="6"/>
+      <c r="E12" s="6"/>
       <c r="F12" s="1" t="s">
-        <v>57</v>
+        <v>2</v>
       </c>
       <c r="G12" s="1" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7">
-      <c r="A13" s="10">
-        <v>46099</v>
+        <v>88</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" ht="18" customHeight="1">
+      <c r="A13" s="9">
+        <v>46102</v>
       </c>
       <c r="B13" s="1" t="str">
         <f t="shared" si="0"/>
-        <v>Mittwoch</v>
+        <v>TTTT</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="D13" s="1"/>
       <c r="E13" s="1"/>
       <c r="F13" s="1" t="s">
-        <v>9</v>
+        <v>92</v>
       </c>
       <c r="G13" s="1" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="14" spans="1:7">
-      <c r="A14" s="10">
-        <v>46100</v>
+    <row r="14" spans="1:7" ht="18" customHeight="1">
+      <c r="A14" s="9">
+        <v>46103</v>
       </c>
       <c r="B14" s="1" t="str">
         <f t="shared" si="0"/>
-        <v>Donnerstag</v>
+        <v>TTTT</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="D14" s="7"/>
-      <c r="E14" s="7"/>
+        <v>11</v>
+      </c>
+      <c r="D14" s="1"/>
+      <c r="E14" s="1"/>
       <c r="F14" s="1" t="s">
-        <v>2</v>
+        <v>93</v>
       </c>
       <c r="G14" s="1" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7">
-      <c r="A15" s="10">
-        <v>46102</v>
+        <v>87</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" ht="18" customHeight="1">
+      <c r="A15" s="9">
+        <v>46111</v>
       </c>
       <c r="B15" s="1" t="str">
         <f t="shared" si="0"/>
-        <v>Samstag</v>
+        <v>TTTT</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="D15" s="1"/>
       <c r="E15" s="1"/>
       <c r="F15" s="1" t="s">
-        <v>92</v>
+        <v>8</v>
       </c>
       <c r="G15" s="1" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="16" spans="1:7">
-      <c r="A16" s="10">
-        <v>46103</v>
+    <row r="16" spans="1:7" ht="18" customHeight="1">
+      <c r="A16" s="9">
+        <v>46123</v>
       </c>
       <c r="B16" s="1" t="str">
         <f t="shared" si="0"/>
-        <v>Sonntag</v>
+        <v>TTTT</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D16" s="1"/>
+        <v>12</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>54</v>
+      </c>
       <c r="E16" s="1"/>
       <c r="F16" s="1" t="s">
-        <v>93</v>
+        <v>8</v>
       </c>
       <c r="G16" s="1" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="17" spans="1:7">
-      <c r="A17" s="10">
-        <v>46111</v>
+    <row r="17" spans="1:7" ht="18" customHeight="1">
+      <c r="A17" s="9">
+        <v>46123</v>
       </c>
       <c r="B17" s="1" t="str">
         <f t="shared" si="0"/>
-        <v>Montag</v>
+        <v>TTTT</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="D17" s="1"/>
-      <c r="E17" s="1"/>
+        <v>44</v>
+      </c>
+      <c r="D17" s="6"/>
+      <c r="E17" s="6"/>
       <c r="F17" s="1" t="s">
-        <v>8</v>
+        <v>77</v>
       </c>
       <c r="G17" s="1" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7">
-      <c r="A18" s="10">
-        <v>46123</v>
+        <v>88</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" ht="18" customHeight="1">
+      <c r="A18" s="9">
+        <v>46125</v>
       </c>
       <c r="B18" s="1" t="str">
         <f t="shared" si="0"/>
-        <v>Samstag</v>
+        <v>TTTT</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="D18" s="1" t="s">
-        <v>54</v>
-      </c>
+        <v>27</v>
+      </c>
+      <c r="D18" s="1"/>
       <c r="E18" s="1"/>
       <c r="F18" s="1" t="s">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="G18" s="1" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="19" spans="1:7">
-      <c r="A19" s="10">
-        <v>46123</v>
+    <row r="19" spans="1:7" ht="18" customHeight="1">
+      <c r="A19" s="9">
+        <v>46134</v>
       </c>
       <c r="B19" s="1" t="str">
         <f t="shared" si="0"/>
-        <v>Samstag</v>
+        <v>TTTT</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="D19" s="7"/>
-      <c r="E19" s="7"/>
+        <v>14</v>
+      </c>
+      <c r="D19" s="1"/>
+      <c r="E19" s="1"/>
       <c r="F19" s="1" t="s">
-        <v>77</v>
+        <v>59</v>
       </c>
       <c r="G19" s="1" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7">
-      <c r="A20" s="10">
-        <v>46125</v>
+        <v>87</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" ht="18" customHeight="1">
+      <c r="A20" s="9">
+        <v>46136</v>
       </c>
       <c r="B20" s="1" t="str">
         <f t="shared" si="0"/>
-        <v>Montag</v>
+        <v>TTTT</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="D20" s="1"/>
-      <c r="E20" s="1"/>
+        <v>47</v>
+      </c>
+      <c r="D20" s="6"/>
+      <c r="E20" s="6"/>
       <c r="F20" s="1" t="s">
-        <v>13</v>
+        <v>95</v>
       </c>
       <c r="G20" s="1" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="21" spans="1:7">
+    <row r="21" spans="1:7" ht="18" customHeight="1">
       <c r="A21" s="10">
-        <v>46134</v>
-      </c>
-      <c r="B21" s="1" t="str">
+        <v>46137</v>
+      </c>
+      <c r="B21" s="2" t="str">
         <f t="shared" si="0"/>
-        <v>Mittwoch</v>
+        <v>TTTT</v>
       </c>
       <c r="C21" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="D21" s="6"/>
+      <c r="E21" s="6"/>
+      <c r="F21" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="G21" s="1" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" ht="18" customHeight="1">
+      <c r="A22" s="10">
+        <v>46137</v>
+      </c>
+      <c r="B22" s="2" t="str">
+        <f t="shared" si="0"/>
+        <v>TTTT</v>
+      </c>
+      <c r="C22" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="D22" s="6"/>
+      <c r="E22" s="6"/>
+      <c r="F22" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G22" s="1" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" ht="18" customHeight="1">
+      <c r="A23" s="9">
+        <v>46139</v>
+      </c>
+      <c r="B23" s="1" t="str">
+        <f t="shared" si="0"/>
+        <v>TTTT</v>
+      </c>
+      <c r="C23" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="D21" s="1"/>
-      <c r="E21" s="1"/>
-      <c r="F21" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="G21" s="1" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="22" spans="1:7">
-      <c r="A22" s="10">
-        <v>46136</v>
-      </c>
-      <c r="B22" s="1" t="str">
+      <c r="D23" s="1"/>
+      <c r="E23" s="1"/>
+      <c r="F23" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="G23" s="1" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" ht="18" customHeight="1">
+      <c r="A24" s="9">
+        <v>46143</v>
+      </c>
+      <c r="B24" s="1" t="str">
         <f t="shared" si="0"/>
-        <v>Freitag</v>
-      </c>
-      <c r="C22" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="D22" s="7"/>
-      <c r="E22" s="7"/>
-      <c r="F22" s="1" t="s">
+        <v>TTTT</v>
+      </c>
+      <c r="C24" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="D24" s="6"/>
+      <c r="E24" s="6"/>
+      <c r="F24" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="G22" s="1" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7" ht="29">
-      <c r="A23" s="11">
-        <v>46137</v>
-      </c>
-      <c r="B23" s="2" t="str">
-        <f t="shared" si="0"/>
-        <v>Samstag</v>
-      </c>
-      <c r="C23" s="1" t="s">
-        <v>101</v>
-      </c>
-      <c r="D23" s="7"/>
-      <c r="E23" s="7"/>
-      <c r="F23" s="2" t="s">
-        <v>95</v>
-      </c>
-      <c r="G23" s="1" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="24" spans="1:7" ht="29">
-      <c r="A24" s="11">
-        <v>46137</v>
-      </c>
-      <c r="B24" s="2" t="str">
-        <f t="shared" si="0"/>
-        <v>Samstag</v>
-      </c>
-      <c r="C24" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="D24" s="7"/>
-      <c r="E24" s="7"/>
-      <c r="F24" s="2" t="s">
-        <v>16</v>
-      </c>
       <c r="G24" s="1" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="25" spans="1:7">
-      <c r="A25" s="10">
-        <v>46139</v>
+    <row r="25" spans="1:7" ht="18" customHeight="1">
+      <c r="A25" s="9">
+        <v>46148</v>
       </c>
       <c r="B25" s="1" t="str">
         <f t="shared" si="0"/>
-        <v>Montag</v>
+        <v>TTTT</v>
       </c>
       <c r="C25" s="1" t="s">
         <v>14</v>
@@ -1570,165 +1547,165 @@
       <c r="D25" s="1"/>
       <c r="E25" s="1"/>
       <c r="F25" s="1" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="G25" s="1" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="26" spans="1:7">
+    <row r="26" spans="1:7" ht="18" customHeight="1">
       <c r="A26" s="10">
-        <v>46143</v>
-      </c>
-      <c r="B26" s="1" t="str">
+        <v>46151</v>
+      </c>
+      <c r="B26" s="2" t="str">
         <f t="shared" si="0"/>
-        <v>Freitag</v>
+        <v>TTTT</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="D26" s="7"/>
-      <c r="E26" s="7"/>
-      <c r="F26" s="1" t="s">
-        <v>95</v>
-      </c>
-      <c r="G26" s="1" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="27" spans="1:7">
-      <c r="A27" s="10">
-        <v>46148</v>
+        <v>70</v>
+      </c>
+      <c r="D26" s="6"/>
+      <c r="E26" s="6"/>
+      <c r="F26" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G26" s="2" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" ht="18" customHeight="1">
+      <c r="A27" s="9">
+        <v>46151</v>
       </c>
       <c r="B27" s="1" t="str">
         <f t="shared" si="0"/>
-        <v>Mittwoch</v>
+        <v>TTTT</v>
       </c>
       <c r="C27" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="D27" s="6"/>
+      <c r="E27" s="6"/>
+      <c r="F27" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="G27" s="1" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" ht="18" customHeight="1">
+      <c r="A28" s="9">
+        <v>46153</v>
+      </c>
+      <c r="B28" s="1" t="str">
+        <f t="shared" si="0"/>
+        <v>TTTT</v>
+      </c>
+      <c r="C28" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="D27" s="1"/>
-      <c r="E27" s="1"/>
-      <c r="F27" s="1" t="s">
+      <c r="D28" s="1"/>
+      <c r="E28" s="1"/>
+      <c r="F28" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="G27" s="1" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7" ht="29">
-      <c r="A28" s="11">
-        <v>46151</v>
-      </c>
-      <c r="B28" s="2" t="str">
-        <f t="shared" si="0"/>
-        <v>Samstag</v>
-      </c>
-      <c r="C28" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="D28" s="7"/>
-      <c r="E28" s="7"/>
-      <c r="F28" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="G28" s="2" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="29" spans="1:7">
-      <c r="A29" s="10">
-        <v>46151</v>
+      <c r="G28" s="1" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" ht="18" customHeight="1">
+      <c r="A29" s="9">
+        <v>46158</v>
       </c>
       <c r="B29" s="1" t="str">
         <f t="shared" si="0"/>
-        <v>Samstag</v>
+        <v>TTTT</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="D29" s="7"/>
-      <c r="E29" s="7"/>
+        <v>53</v>
+      </c>
+      <c r="D29" s="6"/>
+      <c r="E29" s="6"/>
       <c r="F29" s="1" t="s">
-        <v>73</v>
+        <v>52</v>
       </c>
       <c r="G29" s="1" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="30" spans="1:7">
-      <c r="A30" s="10">
-        <v>46153</v>
+    <row r="30" spans="1:7" ht="18" customHeight="1">
+      <c r="A30" s="9">
+        <v>46162</v>
       </c>
       <c r="B30" s="1" t="str">
         <f t="shared" si="0"/>
-        <v>Montag</v>
+        <v>TTTT</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D30" s="1"/>
       <c r="E30" s="1"/>
       <c r="F30" s="1" t="s">
-        <v>21</v>
+        <v>8</v>
       </c>
       <c r="G30" s="1" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="31" spans="1:7">
-      <c r="A31" s="10">
-        <v>46158</v>
+    <row r="31" spans="1:7" ht="18" customHeight="1">
+      <c r="A31" s="9">
+        <v>46171</v>
       </c>
       <c r="B31" s="1" t="str">
         <f t="shared" si="0"/>
-        <v>Samstag</v>
+        <v>TTTT</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="D31" s="7"/>
-      <c r="E31" s="7"/>
+        <v>15</v>
+      </c>
+      <c r="D31" s="6"/>
+      <c r="E31" s="6"/>
       <c r="F31" s="1" t="s">
-        <v>52</v>
+        <v>18</v>
       </c>
       <c r="G31" s="1" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="32" spans="1:7">
-      <c r="A32" s="10">
-        <v>46162</v>
+    <row r="32" spans="1:7" ht="18" customHeight="1">
+      <c r="A32" s="9">
+        <v>46172</v>
       </c>
       <c r="B32" s="1" t="str">
         <f t="shared" si="0"/>
-        <v>Mittwoch</v>
+        <v>TTTT</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="D32" s="1"/>
-      <c r="E32" s="1"/>
+        <v>38</v>
+      </c>
+      <c r="D32" s="6"/>
+      <c r="E32" s="6"/>
       <c r="F32" s="1" t="s">
-        <v>8</v>
+        <v>18</v>
       </c>
       <c r="G32" s="1" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="33" spans="1:7">
-      <c r="A33" s="10">
-        <v>46171</v>
+    <row r="33" spans="1:7" ht="18" customHeight="1">
+      <c r="A33" s="9">
+        <v>46173</v>
       </c>
       <c r="B33" s="1" t="str">
         <f t="shared" si="0"/>
-        <v>Freitag</v>
+        <v>TTTT</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="D33" s="7"/>
-      <c r="E33" s="7"/>
+        <v>38</v>
+      </c>
+      <c r="D33" s="6"/>
+      <c r="E33" s="6"/>
       <c r="F33" s="1" t="s">
         <v>18</v>
       </c>
@@ -1736,235 +1713,235 @@
         <v>87</v>
       </c>
     </row>
-    <row r="34" spans="1:7">
-      <c r="A34" s="10">
-        <v>46172</v>
+    <row r="34" spans="1:7" ht="18" customHeight="1">
+      <c r="A34" s="9">
+        <v>46179</v>
       </c>
       <c r="B34" s="1" t="str">
         <f t="shared" si="0"/>
-        <v>Samstag</v>
+        <v>TTTT</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="D34" s="7"/>
-      <c r="E34" s="7"/>
+        <v>12</v>
+      </c>
+      <c r="D34" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="E34" s="1"/>
       <c r="F34" s="1" t="s">
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="G34" s="1" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="35" spans="1:7">
-      <c r="A35" s="10">
-        <v>46173</v>
+    <row r="35" spans="1:7" ht="18" customHeight="1">
+      <c r="A35" s="9">
+        <v>46183</v>
       </c>
       <c r="B35" s="1" t="str">
-        <f t="shared" si="0"/>
-        <v>Sonntag</v>
+        <f t="shared" ref="B35:B66" si="1">TEXT(A35,"TTTT")</f>
+        <v>TTTT</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="D35" s="7"/>
-      <c r="E35" s="7"/>
+        <v>14</v>
+      </c>
+      <c r="D35" s="1"/>
+      <c r="E35" s="1"/>
       <c r="F35" s="1" t="s">
-        <v>18</v>
+        <v>74</v>
       </c>
       <c r="G35" s="1" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="36" spans="1:7">
-      <c r="A36" s="10">
-        <v>46179</v>
+    <row r="36" spans="1:7" ht="18" customHeight="1">
+      <c r="A36" s="9">
+        <v>46185</v>
       </c>
       <c r="B36" s="1" t="str">
-        <f t="shared" si="0"/>
-        <v>Samstag</v>
+        <f t="shared" si="1"/>
+        <v>TTTT</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="D36" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="E36" s="1"/>
+        <v>15</v>
+      </c>
+      <c r="D36" s="6"/>
+      <c r="E36" s="6"/>
       <c r="F36" s="1" t="s">
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="G36" s="1" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="37" spans="1:7">
+    <row r="37" spans="1:7" ht="18" customHeight="1">
       <c r="A37" s="10">
-        <v>46183</v>
-      </c>
-      <c r="B37" s="1" t="str">
-        <f t="shared" ref="B37:B68" si="1">TEXT(A37,"TTTT")</f>
-        <v>Mittwoch</v>
+        <v>46186</v>
+      </c>
+      <c r="B37" s="2" t="str">
+        <f t="shared" si="1"/>
+        <v>TTTT</v>
       </c>
       <c r="C37" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="D37" s="6"/>
+      <c r="E37" s="6"/>
+      <c r="F37" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="G37" s="1" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" ht="18" customHeight="1">
+      <c r="A38" s="9">
+        <v>46186</v>
+      </c>
+      <c r="B38" s="1" t="str">
+        <f t="shared" si="1"/>
+        <v>TTTT</v>
+      </c>
+      <c r="C38" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="D38" s="6"/>
+      <c r="E38" s="6"/>
+      <c r="F38" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="G38" s="1" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" ht="18" customHeight="1">
+      <c r="A39" s="9">
+        <v>46187</v>
+      </c>
+      <c r="B39" s="1" t="str">
+        <f t="shared" si="1"/>
+        <v>TTTT</v>
+      </c>
+      <c r="C39" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="D39" s="6"/>
+      <c r="E39" s="6"/>
+      <c r="F39" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="G39" s="1" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" ht="18" customHeight="1">
+      <c r="A40" s="9">
+        <v>46190</v>
+      </c>
+      <c r="B40" s="1" t="str">
+        <f t="shared" si="1"/>
+        <v>TTTT</v>
+      </c>
+      <c r="C40" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="D37" s="1"/>
-      <c r="E37" s="1"/>
-      <c r="F37" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="G37" s="1" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="38" spans="1:7">
-      <c r="A38" s="10">
-        <v>46185</v>
-      </c>
-      <c r="B38" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v>Freitag</v>
-      </c>
-      <c r="C38" s="1" t="s">
+      <c r="D40" s="1"/>
+      <c r="E40" s="1"/>
+      <c r="F40" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="G40" s="1" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" ht="18" customHeight="1">
+      <c r="A41" s="10">
+        <v>46192</v>
+      </c>
+      <c r="B41" s="1" t="str">
+        <f t="shared" si="1"/>
+        <v>TTTT</v>
+      </c>
+      <c r="C41" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="D38" s="7"/>
-      <c r="E38" s="7"/>
-      <c r="F38" s="1" t="s">
+      <c r="D41" s="6"/>
+      <c r="E41" s="6"/>
+      <c r="F41" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="G38" s="1" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="39" spans="1:7" ht="29">
-      <c r="A39" s="11">
-        <v>46186</v>
-      </c>
-      <c r="B39" s="2" t="str">
-        <f t="shared" si="1"/>
-        <v>Samstag</v>
-      </c>
-      <c r="C39" s="1" t="s">
+      <c r="G41" s="1" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" ht="18" customHeight="1">
+      <c r="A42" s="10">
+        <v>46193</v>
+      </c>
+      <c r="B42" s="2" t="str">
+        <f t="shared" si="1"/>
+        <v>TTTT</v>
+      </c>
+      <c r="C42" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="D39" s="7"/>
-      <c r="E39" s="7"/>
-      <c r="F39" s="2" t="s">
+      <c r="D42" s="6"/>
+      <c r="E42" s="6"/>
+      <c r="F42" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="G39" s="1" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="40" spans="1:7">
-      <c r="A40" s="10">
-        <v>46186</v>
-      </c>
-      <c r="B40" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v>Samstag</v>
-      </c>
-      <c r="C40" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="D40" s="7"/>
-      <c r="E40" s="7"/>
-      <c r="F40" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="G40" s="1" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="41" spans="1:7">
-      <c r="A41" s="10">
-        <v>46187</v>
-      </c>
-      <c r="B41" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v>Sonntag</v>
-      </c>
-      <c r="C41" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="D41" s="7"/>
-      <c r="E41" s="7"/>
-      <c r="F41" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="G41" s="1" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="42" spans="1:7">
-      <c r="A42" s="10">
-        <v>46190</v>
-      </c>
-      <c r="B42" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v>Mittwoch</v>
-      </c>
-      <c r="C42" s="1" t="s">
+      <c r="G42" s="1" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7" ht="18" customHeight="1">
+      <c r="A43" s="9">
+        <v>46195</v>
+      </c>
+      <c r="B43" s="1" t="str">
+        <f t="shared" si="1"/>
+        <v>TTTT</v>
+      </c>
+      <c r="C43" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="D42" s="1"/>
-      <c r="E42" s="1"/>
-      <c r="F42" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="G42" s="1" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="43" spans="1:7">
-      <c r="A43" s="11">
-        <v>46192</v>
-      </c>
-      <c r="B43" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v>Freitag</v>
-      </c>
-      <c r="C43" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="D43" s="7"/>
-      <c r="E43" s="7"/>
+      <c r="D43" s="1"/>
+      <c r="E43" s="1"/>
       <c r="F43" s="1" t="s">
-        <v>20</v>
+        <v>62</v>
       </c>
       <c r="G43" s="1" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="44" spans="1:7" ht="29">
-      <c r="A44" s="11">
-        <v>46193</v>
-      </c>
-      <c r="B44" s="2" t="str">
-        <f t="shared" si="1"/>
-        <v>Samstag</v>
+    <row r="44" spans="1:7" ht="18" customHeight="1">
+      <c r="A44" s="9">
+        <v>46196</v>
+      </c>
+      <c r="B44" s="1" t="str">
+        <f t="shared" si="1"/>
+        <v>TTTT</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>90</v>
-      </c>
-      <c r="D44" s="7"/>
-      <c r="E44" s="7"/>
-      <c r="F44" s="2" t="s">
-        <v>20</v>
+        <v>49</v>
+      </c>
+      <c r="D44" s="6"/>
+      <c r="E44" s="6"/>
+      <c r="F44" s="1" t="s">
+        <v>50</v>
       </c>
       <c r="G44" s="1" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="45" spans="1:7">
-      <c r="A45" s="10">
-        <v>46195</v>
+    <row r="45" spans="1:7" ht="18" customHeight="1">
+      <c r="A45" s="9">
+        <v>46204</v>
       </c>
       <c r="B45" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>Montag</v>
+        <v>TTTT</v>
       </c>
       <c r="C45" s="1" t="s">
         <v>14</v>
@@ -1972,121 +1949,121 @@
       <c r="D45" s="1"/>
       <c r="E45" s="1"/>
       <c r="F45" s="1" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="G45" s="1" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="46" spans="1:7">
-      <c r="A46" s="10">
-        <v>46196</v>
+    <row r="46" spans="1:7" ht="18" customHeight="1">
+      <c r="A46" s="9">
+        <v>46209</v>
       </c>
       <c r="B46" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>Dienstag</v>
+        <v>TTTT</v>
       </c>
       <c r="C46" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="D46" s="7"/>
-      <c r="E46" s="7"/>
+        <v>14</v>
+      </c>
+      <c r="D46" s="1"/>
+      <c r="E46" s="1"/>
       <c r="F46" s="1" t="s">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="G46" s="1" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="47" spans="1:7">
-      <c r="A47" s="10">
-        <v>46204</v>
+    <row r="47" spans="1:7" ht="18" customHeight="1">
+      <c r="A47" s="9">
+        <v>46214</v>
       </c>
       <c r="B47" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>Mittwoch</v>
+        <v>TTTT</v>
       </c>
       <c r="C47" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="D47" s="1"/>
+        <v>12</v>
+      </c>
+      <c r="D47" s="1" t="s">
+        <v>54</v>
+      </c>
       <c r="E47" s="1"/>
       <c r="F47" s="1" t="s">
-        <v>67</v>
+        <v>8</v>
       </c>
       <c r="G47" s="1" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="48" spans="1:7">
-      <c r="A48" s="10">
-        <v>46209</v>
+    <row r="48" spans="1:7" ht="18" customHeight="1">
+      <c r="A48" s="9">
+        <v>46219</v>
       </c>
       <c r="B48" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>Montag</v>
+        <v>TTTT</v>
       </c>
       <c r="C48" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="D48" s="1"/>
-      <c r="E48" s="1"/>
+      <c r="D48" s="6"/>
+      <c r="E48" s="6"/>
       <c r="F48" s="1" t="s">
-        <v>60</v>
+        <v>79</v>
       </c>
       <c r="G48" s="1" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="49" spans="1:7">
-      <c r="A49" s="10">
-        <v>46214</v>
+    <row r="49" spans="1:7" ht="18" customHeight="1">
+      <c r="A49" s="9">
+        <v>46244</v>
       </c>
       <c r="B49" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>Samstag</v>
+        <v>TTTT</v>
       </c>
       <c r="C49" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="D49" s="1" t="s">
-        <v>54</v>
-      </c>
+        <v>14</v>
+      </c>
+      <c r="D49" s="1"/>
       <c r="E49" s="1"/>
       <c r="F49" s="1" t="s">
-        <v>8</v>
+        <v>23</v>
       </c>
       <c r="G49" s="1" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="50" spans="1:7">
-      <c r="A50" s="10">
-        <v>46219</v>
+    <row r="50" spans="1:7" ht="18" customHeight="1">
+      <c r="A50" s="9">
+        <v>46248</v>
       </c>
       <c r="B50" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>Donnerstag</v>
+        <v>TTTT</v>
       </c>
       <c r="C50" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="D50" s="7"/>
-      <c r="E50" s="7"/>
+        <v>61</v>
+      </c>
+      <c r="D50" s="6"/>
+      <c r="E50" s="6"/>
       <c r="F50" s="1" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="G50" s="1" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="51" spans="1:7">
-      <c r="A51" s="10">
-        <v>46244</v>
+    <row r="51" spans="1:7" ht="18" customHeight="1">
+      <c r="A51" s="9">
+        <v>46251</v>
       </c>
       <c r="B51" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>Montag</v>
+        <v>TTTT</v>
       </c>
       <c r="C51" s="1" t="s">
         <v>14</v>
@@ -2094,139 +2071,139 @@
       <c r="D51" s="1"/>
       <c r="E51" s="1"/>
       <c r="F51" s="1" t="s">
-        <v>23</v>
+        <v>72</v>
       </c>
       <c r="G51" s="1" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="52" spans="1:7">
-      <c r="A52" s="10">
-        <v>46248</v>
+    <row r="52" spans="1:7" ht="18" customHeight="1">
+      <c r="A52" s="9">
+        <v>46253</v>
       </c>
       <c r="B52" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>Freitag</v>
+        <v>TTTT</v>
       </c>
       <c r="C52" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="D52" s="7"/>
-      <c r="E52" s="7"/>
+        <v>24</v>
+      </c>
+      <c r="D52" s="1"/>
+      <c r="E52" s="1"/>
       <c r="F52" s="1" t="s">
-        <v>76</v>
+        <v>25</v>
       </c>
       <c r="G52" s="1" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="53" spans="1:7">
-      <c r="A53" s="10">
-        <v>46251</v>
+    <row r="53" spans="1:7" ht="18" customHeight="1">
+      <c r="A53" s="9">
+        <v>46256</v>
       </c>
       <c r="B53" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>Montag</v>
+        <v>TTTT</v>
       </c>
       <c r="C53" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="D53" s="6"/>
+      <c r="E53" s="6"/>
+      <c r="F53" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="G53" s="1" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="54" spans="1:7" ht="18" customHeight="1">
+      <c r="A54" s="9">
+        <v>46258</v>
+      </c>
+      <c r="B54" s="1" t="str">
+        <f t="shared" si="1"/>
+        <v>TTTT</v>
+      </c>
+      <c r="C54" s="1" t="s">
         <v>14</v>
-      </c>
-      <c r="D53" s="1"/>
-      <c r="E53" s="1"/>
-      <c r="F53" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="G53" s="1" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="54" spans="1:7">
-      <c r="A54" s="10">
-        <v>46253</v>
-      </c>
-      <c r="B54" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v>Mittwoch</v>
-      </c>
-      <c r="C54" s="1" t="s">
-        <v>24</v>
       </c>
       <c r="D54" s="1"/>
       <c r="E54" s="1"/>
       <c r="F54" s="1" t="s">
-        <v>25</v>
+        <v>75</v>
       </c>
       <c r="G54" s="1" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="55" spans="1:7">
-      <c r="A55" s="10">
-        <v>46256</v>
+    <row r="55" spans="1:7" ht="18" customHeight="1">
+      <c r="A55" s="9">
+        <v>46262</v>
       </c>
       <c r="B55" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>Samstag</v>
+        <v>TTTT</v>
       </c>
       <c r="C55" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="D55" s="7"/>
-      <c r="E55" s="7"/>
+        <v>26</v>
+      </c>
+      <c r="D55" s="6"/>
+      <c r="E55" s="6"/>
       <c r="F55" s="1" t="s">
-        <v>94</v>
+        <v>68</v>
       </c>
       <c r="G55" s="1" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="56" spans="1:7">
-      <c r="A56" s="10">
-        <v>46258</v>
+    <row r="56" spans="1:7" ht="18" customHeight="1">
+      <c r="A56" s="9">
+        <v>46267</v>
       </c>
       <c r="B56" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>Montag</v>
+        <v>TTTT</v>
       </c>
       <c r="C56" s="1" t="s">
-        <v>14</v>
+        <v>27</v>
       </c>
       <c r="D56" s="1"/>
       <c r="E56" s="1"/>
       <c r="F56" s="1" t="s">
-        <v>75</v>
+        <v>8</v>
       </c>
       <c r="G56" s="1" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="57" spans="1:7">
-      <c r="A57" s="10">
-        <v>46262</v>
+    <row r="57" spans="1:7" ht="18" customHeight="1">
+      <c r="A57" s="9">
+        <v>46272</v>
       </c>
       <c r="B57" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>Freitag</v>
+        <v>TTTT</v>
       </c>
       <c r="C57" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="D57" s="7"/>
-      <c r="E57" s="7"/>
+        <v>27</v>
+      </c>
+      <c r="D57" s="1"/>
+      <c r="E57" s="1"/>
       <c r="F57" s="1" t="s">
-        <v>68</v>
+        <v>8</v>
       </c>
       <c r="G57" s="1" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="58" spans="1:7">
-      <c r="A58" s="10">
-        <v>46267</v>
+    <row r="58" spans="1:7" ht="18" customHeight="1">
+      <c r="A58" s="9">
+        <v>46279</v>
       </c>
       <c r="B58" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>Mittwoch</v>
+        <v>TTTT</v>
       </c>
       <c r="C58" s="1" t="s">
         <v>27</v>
@@ -2234,19 +2211,19 @@
       <c r="D58" s="1"/>
       <c r="E58" s="1"/>
       <c r="F58" s="1" t="s">
-        <v>8</v>
+        <v>28</v>
       </c>
       <c r="G58" s="1" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="59" spans="1:7">
-      <c r="A59" s="10">
-        <v>46272</v>
+    <row r="59" spans="1:7" ht="18" customHeight="1">
+      <c r="A59" s="9">
+        <v>46288</v>
       </c>
       <c r="B59" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>Montag</v>
+        <v>TTTT</v>
       </c>
       <c r="C59" s="1" t="s">
         <v>27</v>
@@ -2254,585 +2231,573 @@
       <c r="D59" s="1"/>
       <c r="E59" s="1"/>
       <c r="F59" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="G59" s="1" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="60" spans="1:7" ht="18" customHeight="1">
+      <c r="A60" s="9">
+        <v>46290</v>
+      </c>
+      <c r="B60" s="1" t="str">
+        <f t="shared" si="1"/>
+        <v>TTTT</v>
+      </c>
+      <c r="C60" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D60" s="6"/>
+      <c r="E60" s="6"/>
+      <c r="F60" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="G60" s="1" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="61" spans="1:7" ht="18" customHeight="1">
+      <c r="A61" s="10">
+        <v>46291</v>
+      </c>
+      <c r="B61" s="2" t="str">
+        <f t="shared" si="1"/>
+        <v>TTTT</v>
+      </c>
+      <c r="C61" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="D61" s="6"/>
+      <c r="E61" s="6"/>
+      <c r="F61" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="G61" s="2" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="62" spans="1:7" ht="18" customHeight="1">
+      <c r="A62" s="9">
+        <v>46291</v>
+      </c>
+      <c r="B62" s="1" t="str">
+        <f t="shared" si="1"/>
+        <v>TTTT</v>
+      </c>
+      <c r="C62" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D62" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="E62" s="1"/>
+      <c r="F62" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="G59" s="1" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="60" spans="1:7">
-      <c r="A60" s="10">
-        <v>46279</v>
-      </c>
-      <c r="B60" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v>Montag</v>
-      </c>
-      <c r="C60" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="D60" s="1"/>
-      <c r="E60" s="1"/>
-      <c r="F60" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="G60" s="1" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="61" spans="1:7">
-      <c r="A61" s="10">
-        <v>46288</v>
-      </c>
-      <c r="B61" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v>Mittwoch</v>
-      </c>
-      <c r="C61" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="D61" s="1"/>
-      <c r="E61" s="1"/>
-      <c r="F61" s="1" t="s">
-        <v>104</v>
-      </c>
-      <c r="G61" s="1" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="62" spans="1:7">
-      <c r="A62" s="10">
-        <v>46290</v>
-      </c>
-      <c r="B62" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v>Freitag</v>
-      </c>
-      <c r="C62" s="1" t="s">
+      <c r="G62" s="1" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="63" spans="1:7" ht="18" customHeight="1">
+      <c r="A63" s="9">
+        <v>46293</v>
+      </c>
+      <c r="B63" s="1" t="str">
+        <f t="shared" si="1"/>
+        <v>TTTT</v>
+      </c>
+      <c r="C63" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D63" s="1"/>
+      <c r="E63" s="1"/>
+      <c r="F63" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="G63" s="1" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="64" spans="1:7" ht="18" customHeight="1">
+      <c r="A64" s="9">
+        <v>46297</v>
+      </c>
+      <c r="B64" s="1" t="str">
+        <f t="shared" si="1"/>
+        <v>TTTT</v>
+      </c>
+      <c r="C64" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="D62" s="7"/>
-      <c r="E62" s="7"/>
-      <c r="F62" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="G62" s="1" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="63" spans="1:7" ht="29">
-      <c r="A63" s="11">
-        <v>46291</v>
-      </c>
-      <c r="B63" s="2" t="str">
-        <f t="shared" si="1"/>
-        <v>Samstag</v>
-      </c>
-      <c r="C63" s="1" t="s">
-        <v>89</v>
-      </c>
-      <c r="D63" s="7"/>
-      <c r="E63" s="7"/>
-      <c r="F63" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="G63" s="2" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="64" spans="1:7">
-      <c r="A64" s="10">
-        <v>46291</v>
-      </c>
-      <c r="B64" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v>Samstag</v>
-      </c>
-      <c r="C64" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="D64" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="E64" s="1"/>
+      <c r="D64" s="6"/>
+      <c r="E64" s="6"/>
       <c r="F64" s="1" t="s">
-        <v>8</v>
+        <v>63</v>
       </c>
       <c r="G64" s="1" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="65" spans="1:7">
-      <c r="A65" s="10">
-        <v>46293</v>
+    <row r="65" spans="1:7" ht="18" customHeight="1">
+      <c r="A65" s="9">
+        <v>46298</v>
       </c>
       <c r="B65" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>Montag</v>
+        <v>TTTT</v>
       </c>
       <c r="C65" s="1" t="s">
-        <v>17</v>
+        <v>30</v>
       </c>
       <c r="D65" s="1"/>
       <c r="E65" s="1"/>
       <c r="F65" s="1" t="s">
-        <v>98</v>
+        <v>29</v>
       </c>
       <c r="G65" s="1" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="66" spans="1:7">
-      <c r="A66" s="10">
-        <v>46297</v>
+    <row r="66" spans="1:7" ht="18" customHeight="1">
+      <c r="A66" s="9">
+        <v>46298</v>
       </c>
       <c r="B66" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>Freitag</v>
+        <v>TTTT</v>
       </c>
       <c r="C66" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="D66" s="7"/>
-      <c r="E66" s="7"/>
+        <v>11</v>
+      </c>
+      <c r="D66" s="6"/>
+      <c r="E66" s="6"/>
       <c r="F66" s="1" t="s">
-        <v>63</v>
+        <v>42</v>
       </c>
       <c r="G66" s="1" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="67" spans="1:7">
-      <c r="A67" s="10">
+    <row r="67" spans="1:7" ht="18" customHeight="1">
+      <c r="A67" s="9">
         <v>46298</v>
       </c>
       <c r="B67" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v>Samstag</v>
+        <f t="shared" ref="B67:B98" si="2">TEXT(A67,"TTTT")</f>
+        <v>TTTT</v>
       </c>
       <c r="C67" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="D67" s="1"/>
-      <c r="E67" s="1"/>
+        <v>22</v>
+      </c>
+      <c r="D67" s="6"/>
+      <c r="E67" s="6"/>
       <c r="F67" s="1" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="G67" s="1" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="68" spans="1:7">
-      <c r="A68" s="10">
+    <row r="68" spans="1:7" ht="18" customHeight="1">
+      <c r="A68" s="9">
         <v>46298</v>
       </c>
       <c r="B68" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v>Samstag</v>
-      </c>
-      <c r="C68" s="1" t="s">
+        <f t="shared" si="2"/>
+        <v>TTTT</v>
+      </c>
+      <c r="C68" s="8" t="s">
+        <v>99</v>
+      </c>
+      <c r="D68" s="6"/>
+      <c r="E68" s="6"/>
+      <c r="F68" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="G68" s="1" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="69" spans="1:7" ht="18" customHeight="1">
+      <c r="A69" s="9">
+        <v>46299</v>
+      </c>
+      <c r="B69" s="1" t="str">
+        <f t="shared" si="2"/>
+        <v>TTTT</v>
+      </c>
+      <c r="C69" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D68" s="7"/>
-      <c r="E68" s="7"/>
-      <c r="F68" s="1" t="s">
+      <c r="D69" s="6"/>
+      <c r="E69" s="6"/>
+      <c r="F69" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="G68" s="1" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="69" spans="1:7">
-      <c r="A69" s="10">
-        <v>46298</v>
-      </c>
-      <c r="B69" s="1" t="str">
-        <f t="shared" ref="B69:B100" si="2">TEXT(A69,"TTTT")</f>
-        <v>Samstag</v>
-      </c>
-      <c r="C69" s="1" t="s">
+      <c r="G69" s="1" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="70" spans="1:7" ht="18" customHeight="1">
+      <c r="A70" s="9">
+        <v>46302</v>
+      </c>
+      <c r="B70" s="1" t="str">
+        <f t="shared" si="2"/>
+        <v>TTTT</v>
+      </c>
+      <c r="C70" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D70" s="1"/>
+      <c r="E70" s="1"/>
+      <c r="F70" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="G70" s="1" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="71" spans="1:7" ht="18" customHeight="1">
+      <c r="A71" s="10">
+        <v>46305</v>
+      </c>
+      <c r="B71" s="12" t="str">
+        <f t="shared" si="2"/>
+        <v>TTTT</v>
+      </c>
+      <c r="C71" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="D71" s="6"/>
+      <c r="E71" s="6"/>
+      <c r="F71" s="12" t="s">
+        <v>80</v>
+      </c>
+      <c r="G71" s="2" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="72" spans="1:7" ht="18" customHeight="1">
+      <c r="A72" s="9">
+        <v>46306</v>
+      </c>
+      <c r="B72" s="1" t="str">
+        <f t="shared" si="2"/>
+        <v>TTTT</v>
+      </c>
+      <c r="C72" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="D72" s="6"/>
+      <c r="E72" s="6"/>
+      <c r="F72" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="G72" s="1" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="73" spans="1:7" ht="18" customHeight="1">
+      <c r="A73" s="9">
+        <v>46307</v>
+      </c>
+      <c r="B73" s="1" t="str">
+        <f t="shared" si="2"/>
+        <v>TTTT</v>
+      </c>
+      <c r="C73" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D73" s="1"/>
+      <c r="E73" s="1"/>
+      <c r="F73" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="G73" s="1" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="74" spans="1:7" ht="18" customHeight="1">
+      <c r="A74" s="9">
+        <v>46312</v>
+      </c>
+      <c r="B74" s="1" t="str">
+        <f t="shared" si="2"/>
+        <v>TTTT</v>
+      </c>
+      <c r="C74" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D74" s="6"/>
+      <c r="E74" s="6"/>
+      <c r="F74" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="G74" s="1" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="75" spans="1:7" ht="18" customHeight="1">
+      <c r="A75" s="9">
+        <v>46313</v>
+      </c>
+      <c r="B75" s="1" t="str">
+        <f t="shared" si="2"/>
+        <v>TTTT</v>
+      </c>
+      <c r="C75" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="D69" s="7"/>
-      <c r="E69" s="7"/>
-      <c r="F69" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="G69" s="1" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="70" spans="1:7">
-      <c r="A70" s="10">
-        <v>46298</v>
-      </c>
-      <c r="B70" s="1" t="str">
-        <f t="shared" si="2"/>
-        <v>Samstag</v>
-      </c>
-      <c r="C70" s="9" t="s">
-        <v>99</v>
-      </c>
-      <c r="D70" s="7"/>
-      <c r="E70" s="7"/>
-      <c r="F70" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="G70" s="1" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="71" spans="1:7">
-      <c r="A71" s="10">
-        <v>46299</v>
-      </c>
-      <c r="B71" s="1" t="str">
-        <f t="shared" si="2"/>
-        <v>Sonntag</v>
-      </c>
-      <c r="C71" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D71" s="7"/>
-      <c r="E71" s="7"/>
-      <c r="F71" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="G71" s="1" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="72" spans="1:7">
-      <c r="A72" s="10">
-        <v>46302</v>
-      </c>
-      <c r="B72" s="1" t="str">
-        <f t="shared" si="2"/>
-        <v>Mittwoch</v>
-      </c>
-      <c r="C72" s="1" t="s">
+      <c r="D75" s="6"/>
+      <c r="E75" s="6"/>
+      <c r="F75" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="G75" s="1" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="76" spans="1:7" ht="18" customHeight="1">
+      <c r="A76" s="10">
+        <v>46316</v>
+      </c>
+      <c r="B76" s="1" t="str">
+        <f t="shared" si="2"/>
+        <v>TTTT</v>
+      </c>
+      <c r="C76" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="D72" s="1"/>
-      <c r="E72" s="1"/>
-      <c r="F72" s="1" t="s">
+      <c r="D76" s="1"/>
+      <c r="E76" s="1"/>
+      <c r="F76" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="G72" s="1" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="73" spans="1:7" ht="29">
-      <c r="A73" s="11">
-        <v>46305</v>
-      </c>
-      <c r="B73" s="13" t="str">
-        <f t="shared" si="2"/>
-        <v>Samstag</v>
-      </c>
-      <c r="C73" s="1" t="s">
-        <v>100</v>
-      </c>
-      <c r="D73" s="7"/>
-      <c r="E73" s="7"/>
-      <c r="F73" s="13" t="s">
-        <v>80</v>
-      </c>
-      <c r="G73" s="2" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="74" spans="1:7">
-      <c r="A74" s="10">
-        <v>46306</v>
-      </c>
-      <c r="B74" s="1" t="str">
-        <f t="shared" si="2"/>
-        <v>Sonntag</v>
-      </c>
-      <c r="C74" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="D74" s="7"/>
-      <c r="E74" s="7"/>
-      <c r="F74" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="G74" s="1" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="75" spans="1:7">
-      <c r="A75" s="10">
-        <v>46307</v>
-      </c>
-      <c r="B75" s="1" t="str">
-        <f t="shared" si="2"/>
-        <v>Montag</v>
-      </c>
-      <c r="C75" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="D75" s="1"/>
-      <c r="E75" s="1"/>
-      <c r="F75" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="G75" s="1" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="76" spans="1:7">
-      <c r="A76" s="10">
-        <v>46312</v>
-      </c>
-      <c r="B76" s="1" t="str">
-        <f t="shared" si="2"/>
-        <v>Samstag</v>
-      </c>
-      <c r="C76" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D76" s="7"/>
-      <c r="E76" s="7"/>
-      <c r="F76" s="1" t="s">
+      <c r="G76" s="1" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="77" spans="1:7" ht="18" customHeight="1">
+      <c r="A77" s="10">
+        <v>46319</v>
+      </c>
+      <c r="B77" s="2" t="str">
+        <f t="shared" si="2"/>
+        <v>TTTT</v>
+      </c>
+      <c r="C77" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="D77" s="6"/>
+      <c r="E77" s="6"/>
+      <c r="F77" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="G76" s="1" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="77" spans="1:7">
-      <c r="A77" s="10">
-        <v>46313</v>
-      </c>
-      <c r="B77" s="1" t="str">
-        <f t="shared" si="2"/>
-        <v>Sonntag</v>
-      </c>
-      <c r="C77" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="D77" s="7"/>
-      <c r="E77" s="7"/>
-      <c r="F77" s="1" t="s">
-        <v>86</v>
-      </c>
-      <c r="G77" s="1" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="78" spans="1:7">
-      <c r="A78" s="11">
-        <v>46316</v>
-      </c>
-      <c r="B78" s="1" t="str">
-        <f t="shared" si="2"/>
-        <v>Mittwoch</v>
+      <c r="G77" s="2" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="78" spans="1:7" ht="18" customHeight="1">
+      <c r="A78" s="10">
+        <v>46320</v>
+      </c>
+      <c r="B78" s="2" t="str">
+        <f t="shared" si="2"/>
+        <v>TTTT</v>
       </c>
       <c r="C78" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="D78" s="1"/>
-      <c r="E78" s="1"/>
-      <c r="F78" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="G78" s="1" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="79" spans="1:7" ht="29">
-      <c r="A79" s="11">
-        <v>46319</v>
-      </c>
-      <c r="B79" s="2" t="str">
-        <f t="shared" si="2"/>
-        <v>Samstag</v>
+        <v>103</v>
+      </c>
+      <c r="D78" s="6"/>
+      <c r="E78" s="6"/>
+      <c r="F78" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="G78" s="2" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="79" spans="1:7" ht="18" customHeight="1">
+      <c r="A79" s="9">
+        <v>46323</v>
+      </c>
+      <c r="B79" s="1" t="str">
+        <f t="shared" si="2"/>
+        <v>TTTT</v>
       </c>
       <c r="C79" s="1" t="s">
-        <v>91</v>
-      </c>
-      <c r="D79" s="7"/>
-      <c r="E79" s="7"/>
-      <c r="F79" s="2" t="s">
-        <v>102</v>
-      </c>
-      <c r="G79" s="2" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="80" spans="1:7">
-      <c r="A80" s="11">
-        <v>46320</v>
-      </c>
-      <c r="B80" s="2" t="str">
-        <f t="shared" si="2"/>
-        <v>Sonntag</v>
+        <v>64</v>
+      </c>
+      <c r="D79" s="1"/>
+      <c r="E79" s="1"/>
+      <c r="F79" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="G79" s="1" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="80" spans="1:7" ht="18" customHeight="1">
+      <c r="A80" s="9">
+        <v>46326</v>
+      </c>
+      <c r="B80" s="1" t="str">
+        <f t="shared" si="2"/>
+        <v>TTTT</v>
       </c>
       <c r="C80" s="1" t="s">
-        <v>103</v>
-      </c>
-      <c r="D80" s="7"/>
-      <c r="E80" s="7"/>
-      <c r="F80" s="2" t="s">
-        <v>102</v>
-      </c>
-      <c r="G80" s="2" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="81" spans="1:7">
-      <c r="A81" s="10">
-        <v>46323</v>
+        <v>32</v>
+      </c>
+      <c r="D80" s="1"/>
+      <c r="E80" s="1"/>
+      <c r="F80" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="G80" s="1" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="81" spans="1:7" ht="18" customHeight="1">
+      <c r="A81" s="9">
+        <v>46330</v>
       </c>
       <c r="B81" s="1" t="str">
         <f t="shared" si="2"/>
-        <v>Mittwoch</v>
+        <v>TTTT</v>
       </c>
       <c r="C81" s="1" t="s">
-        <v>64</v>
+        <v>34</v>
       </c>
       <c r="D81" s="1"/>
       <c r="E81" s="1"/>
       <c r="F81" s="1" t="s">
-        <v>58</v>
+        <v>48</v>
       </c>
       <c r="G81" s="1" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="82" spans="1:7">
-      <c r="A82" s="10">
-        <v>46326</v>
+    <row r="82" spans="1:7" ht="18" customHeight="1">
+      <c r="A82" s="9">
+        <v>46337</v>
       </c>
       <c r="B82" s="1" t="str">
         <f t="shared" si="2"/>
-        <v>Samstag</v>
+        <v>TTTT</v>
       </c>
       <c r="C82" s="1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D82" s="1"/>
       <c r="E82" s="1"/>
-      <c r="F82" s="8" t="s">
-        <v>33</v>
+      <c r="F82" s="1" t="s">
+        <v>48</v>
       </c>
       <c r="G82" s="1" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="83" spans="1:7">
-      <c r="A83" s="10">
-        <v>46330</v>
+    <row r="83" spans="1:7" ht="18" customHeight="1" thickBot="1">
+      <c r="A83" s="9">
+        <v>46341</v>
       </c>
       <c r="B83" s="1" t="str">
         <f t="shared" si="2"/>
-        <v>Mittwoch</v>
+        <v>TTTT</v>
       </c>
       <c r="C83" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="D83" s="1"/>
-      <c r="E83" s="1"/>
-      <c r="F83" s="1" t="s">
-        <v>48</v>
+        <v>22</v>
+      </c>
+      <c r="D83" s="6"/>
+      <c r="E83" s="6"/>
+      <c r="F83" s="3" t="s">
+        <v>35</v>
       </c>
       <c r="G83" s="1" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="84" spans="1:7">
-      <c r="A84" s="10">
-        <v>46337</v>
+    <row r="84" spans="1:7" ht="18" customHeight="1">
+      <c r="A84" s="9">
+        <v>46347</v>
       </c>
       <c r="B84" s="1" t="str">
         <f t="shared" si="2"/>
-        <v>Mittwoch</v>
+        <v>TTTT</v>
       </c>
       <c r="C84" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="D84" s="1"/>
-      <c r="E84" s="1"/>
-      <c r="F84" s="1" t="s">
-        <v>48</v>
+        <v>96</v>
+      </c>
+      <c r="D84" s="6" t="s">
+        <v>65</v>
+      </c>
+      <c r="E84" s="6"/>
+      <c r="F84" s="4" t="s">
+        <v>97</v>
       </c>
       <c r="G84" s="1" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="85" spans="1:7" ht="15" thickBot="1">
-      <c r="A85" s="10">
-        <v>46341</v>
+    <row r="85" spans="1:7" ht="18" customHeight="1">
+      <c r="A85" s="9">
+        <v>46349</v>
       </c>
       <c r="B85" s="1" t="str">
         <f t="shared" si="2"/>
-        <v>Sonntag</v>
+        <v>TTTT</v>
       </c>
       <c r="C85" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="D85" s="7"/>
-      <c r="E85" s="7"/>
-      <c r="F85" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
+      </c>
+      <c r="D85" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="E85" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="F85" s="1" t="s">
+        <v>105</v>
       </c>
       <c r="G85" s="1" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="86" spans="1:7">
-      <c r="A86" s="10">
-        <v>46347</v>
-      </c>
+    <row r="86" spans="1:7" ht="18" customHeight="1">
+      <c r="A86" s="9"/>
       <c r="B86" s="1" t="str">
         <f t="shared" si="2"/>
-        <v>Samstag</v>
-      </c>
-      <c r="C86" s="1" t="s">
-        <v>96</v>
-      </c>
-      <c r="D86" s="7" t="s">
-        <v>65</v>
-      </c>
-      <c r="E86" s="7"/>
-      <c r="F86" s="5" t="s">
-        <v>97</v>
-      </c>
+        <v>TTTT</v>
+      </c>
+      <c r="C86" s="1"/>
+      <c r="D86" s="1"/>
+      <c r="E86" s="1"/>
+      <c r="F86" s="1"/>
       <c r="G86" s="1" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="87" spans="1:7">
-      <c r="A87" s="10">
-        <v>46349</v>
-      </c>
+    <row r="87" spans="1:7" ht="18" customHeight="1">
+      <c r="A87" s="9"/>
       <c r="B87" s="1" t="str">
         <f t="shared" si="2"/>
-        <v>Montag</v>
-      </c>
-      <c r="C87" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="D87" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="E87" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="F87" s="1" t="s">
-        <v>105</v>
-      </c>
+        <v>TTTT</v>
+      </c>
+      <c r="C87" s="1"/>
+      <c r="D87" s="1"/>
+      <c r="E87" s="1"/>
+      <c r="F87" s="1"/>
       <c r="G87" s="1" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="88" spans="1:7">
-      <c r="A88" s="10"/>
+    <row r="88" spans="1:7" ht="18" customHeight="1">
+      <c r="A88" s="9"/>
       <c r="B88" s="1" t="str">
         <f t="shared" si="2"/>
-        <v>Samstag</v>
+        <v>TTTT</v>
       </c>
       <c r="C88" s="1"/>
       <c r="D88" s="1"/>
@@ -2842,11 +2807,11 @@
         <v>87</v>
       </c>
     </row>
-    <row r="89" spans="1:7">
-      <c r="A89" s="10"/>
+    <row r="89" spans="1:7" ht="18" customHeight="1">
+      <c r="A89" s="9"/>
       <c r="B89" s="1" t="str">
         <f t="shared" si="2"/>
-        <v>Samstag</v>
+        <v>TTTT</v>
       </c>
       <c r="C89" s="1"/>
       <c r="D89" s="1"/>
@@ -2856,11 +2821,11 @@
         <v>87</v>
       </c>
     </row>
-    <row r="90" spans="1:7">
-      <c r="A90" s="10"/>
+    <row r="90" spans="1:7" ht="18" customHeight="1">
+      <c r="A90" s="9"/>
       <c r="B90" s="1" t="str">
         <f t="shared" si="2"/>
-        <v>Samstag</v>
+        <v>TTTT</v>
       </c>
       <c r="C90" s="1"/>
       <c r="D90" s="1"/>
@@ -2870,11 +2835,11 @@
         <v>87</v>
       </c>
     </row>
-    <row r="91" spans="1:7">
-      <c r="A91" s="10"/>
+    <row r="91" spans="1:7" ht="18" customHeight="1">
+      <c r="A91" s="9"/>
       <c r="B91" s="1" t="str">
         <f t="shared" si="2"/>
-        <v>Samstag</v>
+        <v>TTTT</v>
       </c>
       <c r="C91" s="1"/>
       <c r="D91" s="1"/>
@@ -2884,11 +2849,11 @@
         <v>87</v>
       </c>
     </row>
-    <row r="92" spans="1:7">
-      <c r="A92" s="10"/>
+    <row r="92" spans="1:7" ht="18" customHeight="1">
+      <c r="A92" s="9"/>
       <c r="B92" s="1" t="str">
         <f t="shared" si="2"/>
-        <v>Samstag</v>
+        <v>TTTT</v>
       </c>
       <c r="C92" s="1"/>
       <c r="D92" s="1"/>
@@ -2898,11 +2863,11 @@
         <v>87</v>
       </c>
     </row>
-    <row r="93" spans="1:7">
-      <c r="A93" s="10"/>
+    <row r="93" spans="1:7" ht="18" customHeight="1">
+      <c r="A93" s="9"/>
       <c r="B93" s="1" t="str">
         <f t="shared" si="2"/>
-        <v>Samstag</v>
+        <v>TTTT</v>
       </c>
       <c r="C93" s="1"/>
       <c r="D93" s="1"/>
@@ -2912,11 +2877,11 @@
         <v>87</v>
       </c>
     </row>
-    <row r="94" spans="1:7">
-      <c r="A94" s="10"/>
+    <row r="94" spans="1:7" ht="18" customHeight="1">
+      <c r="A94" s="9"/>
       <c r="B94" s="1" t="str">
         <f t="shared" si="2"/>
-        <v>Samstag</v>
+        <v>TTTT</v>
       </c>
       <c r="C94" s="1"/>
       <c r="D94" s="1"/>
@@ -2926,11 +2891,11 @@
         <v>87</v>
       </c>
     </row>
-    <row r="95" spans="1:7">
-      <c r="A95" s="10"/>
+    <row r="95" spans="1:7" ht="18" customHeight="1">
+      <c r="A95" s="9"/>
       <c r="B95" s="1" t="str">
         <f t="shared" si="2"/>
-        <v>Samstag</v>
+        <v>TTTT</v>
       </c>
       <c r="C95" s="1"/>
       <c r="D95" s="1"/>
@@ -2940,11 +2905,11 @@
         <v>87</v>
       </c>
     </row>
-    <row r="96" spans="1:7">
-      <c r="A96" s="10"/>
+    <row r="96" spans="1:7" ht="18" customHeight="1">
+      <c r="A96" s="9"/>
       <c r="B96" s="1" t="str">
         <f t="shared" si="2"/>
-        <v>Samstag</v>
+        <v>TTTT</v>
       </c>
       <c r="C96" s="1"/>
       <c r="D96" s="1"/>
@@ -2954,11 +2919,11 @@
         <v>87</v>
       </c>
     </row>
-    <row r="97" spans="1:7">
-      <c r="A97" s="10"/>
+    <row r="97" spans="1:7" ht="18" customHeight="1">
+      <c r="A97" s="9"/>
       <c r="B97" s="1" t="str">
         <f t="shared" si="2"/>
-        <v>Samstag</v>
+        <v>TTTT</v>
       </c>
       <c r="C97" s="1"/>
       <c r="D97" s="1"/>
@@ -2968,11 +2933,11 @@
         <v>87</v>
       </c>
     </row>
-    <row r="98" spans="1:7">
-      <c r="A98" s="10"/>
+    <row r="98" spans="1:7" ht="18" customHeight="1">
+      <c r="A98" s="9"/>
       <c r="B98" s="1" t="str">
         <f t="shared" si="2"/>
-        <v>Samstag</v>
+        <v>TTTT</v>
       </c>
       <c r="C98" s="1"/>
       <c r="D98" s="1"/>
@@ -2982,11 +2947,11 @@
         <v>87</v>
       </c>
     </row>
-    <row r="99" spans="1:7">
-      <c r="A99" s="10"/>
+    <row r="99" spans="1:7" ht="18" customHeight="1">
+      <c r="A99" s="9"/>
       <c r="B99" s="1" t="str">
-        <f t="shared" si="2"/>
-        <v>Samstag</v>
+        <f t="shared" ref="B99" si="3">TEXT(A99,"TTTT")</f>
+        <v>TTTT</v>
       </c>
       <c r="C99" s="1"/>
       <c r="D99" s="1"/>
@@ -2996,40 +2961,12 @@
         <v>87</v>
       </c>
     </row>
-    <row r="100" spans="1:7">
-      <c r="A100" s="10"/>
-      <c r="B100" s="1" t="str">
-        <f t="shared" si="2"/>
-        <v>Samstag</v>
-      </c>
-      <c r="C100" s="1"/>
-      <c r="D100" s="1"/>
-      <c r="E100" s="1"/>
-      <c r="F100" s="1"/>
-      <c r="G100" s="1" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="101" spans="1:7">
-      <c r="A101" s="10"/>
-      <c r="B101" s="1" t="str">
-        <f t="shared" ref="B101" si="3">TEXT(A101,"TTTT")</f>
-        <v>Samstag</v>
-      </c>
-      <c r="C101" s="1"/>
-      <c r="D101" s="1"/>
-      <c r="E101" s="1"/>
-      <c r="F101" s="1"/>
-      <c r="G101" s="1" t="s">
-        <v>87</v>
-      </c>
-    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:F1"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G5:G101" xr:uid="{3111A34E-5656-4250-B423-2998DDA71DE5}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G5:G99" xr:uid="{3111A34E-5656-4250-B423-2998DDA71DE5}">
       <formula1>"Ja,Nein"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>